<commit_message>
GEMM CWB results: no ci
</commit_message>
<xml_diff>
--- a/test/gemm/GEMM Partial Acceleration Data.xlsx
+++ b/test/gemm/GEMM Partial Acceleration Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EBC230001\Documents\DARClab\risc_v_asip\test\gemm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7B2826D-D016-4704-AA7D-12DA897109E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18620DBD-FFB0-42A6-91DF-18740F41D112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="8">
   <si>
     <t>Baseline</t>
   </si>
@@ -127,10 +127,10 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -475,49 +475,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="2" customWidth="1"/>
     <col min="3" max="3" width="9.85546875" style="2" customWidth="1"/>
-    <col min="4" max="6" width="9.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="8.28515625" style="2" customWidth="1"/>
+    <col min="5" max="6" width="9.140625" style="2" customWidth="1"/>
     <col min="7" max="7" width="8.7109375" style="2" customWidth="1"/>
     <col min="8" max="8" width="8.140625" style="2" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" style="2" customWidth="1"/>
     <col min="10" max="10" width="8" style="2" customWidth="1"/>
     <col min="11" max="13" width="9.140625" style="2" customWidth="1"/>
     <col min="14" max="14" width="7.140625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="10" style="2" customWidth="1"/>
-    <col min="16" max="19" width="9.140625" style="2" customWidth="1"/>
-    <col min="20" max="20" width="17.5703125" style="2" customWidth="1"/>
-    <col min="21" max="22" width="9.140625" style="2" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="2"/>
+    <col min="15" max="15" width="7.85546875" style="2" customWidth="1"/>
+    <col min="16" max="17" width="9.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="17.5703125" style="2" customWidth="1"/>
+    <col min="19" max="20" width="9.140625" style="2" customWidth="1"/>
+    <col min="21" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
       <c r="E1" s="6"/>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
       <c r="J1" s="7"/>
       <c r="K1" s="7"/>
-      <c r="M1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="6"/>
-    </row>
-    <row r="2" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+    </row>
+    <row r="2" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -530,7 +530,7 @@
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -545,7 +545,7 @@
       <c r="J2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="M2" s="1" t="s">
@@ -555,16 +555,13 @@
         <v>4</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="P2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="P2" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -577,7 +574,7 @@
       <c r="D3" s="1">
         <v>4</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>160149</v>
       </c>
       <c r="G3" s="1">
@@ -592,7 +589,7 @@
       <c r="J3" s="1">
         <v>19</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="3">
         <v>168643</v>
       </c>
       <c r="M3" s="1">
@@ -602,16 +599,13 @@
         <v>0</v>
       </c>
       <c r="O3" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P3" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q3" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="P3" s="3">
+        <v>168643</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G4" s="1">
         <v>1</v>
       </c>
@@ -624,7 +618,7 @@
       <c r="J4" s="1">
         <v>20</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="3">
         <v>304623</v>
       </c>
       <c r="M4" s="1">
@@ -634,16 +628,13 @@
         <v>1</v>
       </c>
       <c r="O4" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P4" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q4" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="P4" s="3">
+        <v>304623</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G5" s="1">
         <v>1</v>
       </c>
@@ -656,7 +647,7 @@
       <c r="J5" s="1">
         <v>20</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="3">
         <v>304913</v>
       </c>
       <c r="M5" s="1">
@@ -666,16 +657,13 @@
         <v>2</v>
       </c>
       <c r="O5" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P5" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q5" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="P5" s="3">
+        <v>304913</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G6" s="1">
         <v>1</v>
       </c>
@@ -688,7 +676,7 @@
       <c r="J6" s="1">
         <v>21</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="3">
         <v>169554</v>
       </c>
       <c r="M6" s="1">
@@ -698,16 +686,13 @@
         <v>4</v>
       </c>
       <c r="O6" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P6" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="P6" s="3">
+        <v>169554</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G7" s="1">
         <v>1</v>
       </c>
@@ -720,7 +705,7 @@
       <c r="J7" s="1">
         <v>19</v>
       </c>
-      <c r="K7" s="4">
+      <c r="K7" s="3">
         <v>168643</v>
       </c>
       <c r="M7" s="1">
@@ -730,16 +715,13 @@
         <v>8</v>
       </c>
       <c r="O7" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P7" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q7" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="P7" s="3">
+        <v>168643</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G8" s="1">
         <v>2</v>
       </c>
@@ -752,7 +734,7 @@
       <c r="J8" s="1">
         <v>11</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="3">
         <v>309365</v>
       </c>
       <c r="M8" s="1">
@@ -762,16 +744,13 @@
         <v>1</v>
       </c>
       <c r="O8" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P8" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q8" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="P8" s="3">
+        <v>309365</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G9" s="1">
         <v>2</v>
       </c>
@@ -784,7 +763,7 @@
       <c r="J9" s="1">
         <v>12</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="3">
         <v>304708</v>
       </c>
       <c r="M9" s="1">
@@ -794,16 +773,13 @@
         <v>0</v>
       </c>
       <c r="O9" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P9" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q9" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P9" s="3">
+        <v>304708</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G10" s="1">
         <v>2</v>
       </c>
@@ -816,7 +792,7 @@
       <c r="J10" s="1">
         <v>12</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="3">
         <v>304666</v>
       </c>
       <c r="M10" s="1">
@@ -826,16 +802,13 @@
         <v>2</v>
       </c>
       <c r="O10" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P10" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q10" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P10" s="3">
+        <v>304666</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G11" s="1">
         <v>2</v>
       </c>
@@ -848,7 +821,7 @@
       <c r="J11" s="1">
         <v>13</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K11" s="3">
         <v>582138</v>
       </c>
       <c r="M11" s="1">
@@ -858,16 +831,13 @@
         <v>4</v>
       </c>
       <c r="O11" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P11" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q11" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="P11" s="3">
+        <v>582138</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G12" s="1">
         <v>2</v>
       </c>
@@ -880,7 +850,7 @@
       <c r="J12" s="1">
         <v>11</v>
       </c>
-      <c r="K12" s="4">
+      <c r="K12" s="3">
         <v>309365</v>
       </c>
       <c r="M12" s="1">
@@ -890,16 +860,13 @@
         <v>8</v>
       </c>
       <c r="O12" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P12" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q12" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+      <c r="P12" s="3">
+        <v>309365</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G13" s="1">
         <v>4</v>
       </c>
@@ -912,7 +879,7 @@
       <c r="J13" s="1">
         <v>8</v>
       </c>
-      <c r="K13" s="4">
+      <c r="K13" s="3">
         <v>862160</v>
       </c>
       <c r="M13" s="1">
@@ -922,16 +889,13 @@
         <v>0</v>
       </c>
       <c r="O13" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P13" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q13" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="P13" s="3">
+        <v>862160</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G14" s="1">
         <v>4</v>
       </c>
@@ -944,7 +908,7 @@
       <c r="J14" s="1">
         <v>12</v>
       </c>
-      <c r="K14" s="4">
+      <c r="K14" s="3">
         <v>304708</v>
       </c>
       <c r="M14" s="1">
@@ -954,16 +918,13 @@
         <v>1</v>
       </c>
       <c r="O14" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P14" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q14" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P14" s="3">
+        <v>304708</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G15" s="1">
         <v>4</v>
       </c>
@@ -976,7 +937,7 @@
       <c r="J15" s="1">
         <v>12</v>
       </c>
-      <c r="K15" s="4">
+      <c r="K15" s="3">
         <v>304666</v>
       </c>
       <c r="M15" s="1">
@@ -986,16 +947,13 @@
         <v>2</v>
       </c>
       <c r="O15" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P15" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q15" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P15" s="3">
+        <v>304666</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="G16" s="1">
         <v>4</v>
       </c>
@@ -1008,7 +966,7 @@
       <c r="J16" s="1">
         <v>9</v>
       </c>
-      <c r="K16" s="4">
+      <c r="K16" s="3">
         <v>997640</v>
       </c>
       <c r="M16" s="1">
@@ -1018,16 +976,13 @@
         <v>4</v>
       </c>
       <c r="O16" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P16" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q16" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="17" spans="7:17" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+      <c r="P16" s="3">
+        <v>997640</v>
+      </c>
+    </row>
+    <row r="17" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G17" s="1">
         <v>4</v>
       </c>
@@ -1040,7 +995,7 @@
       <c r="J17" s="1">
         <v>8</v>
       </c>
-      <c r="K17" s="4">
+      <c r="K17" s="3">
         <v>862160</v>
       </c>
       <c r="M17" s="1">
@@ -1050,16 +1005,13 @@
         <v>8</v>
       </c>
       <c r="O17" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P17" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q17" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="18" spans="7:17" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="P17" s="3">
+        <v>862160</v>
+      </c>
+    </row>
+    <row r="18" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G18" s="1">
         <v>8</v>
       </c>
@@ -1072,7 +1024,7 @@
       <c r="J18" s="1">
         <v>6</v>
       </c>
-      <c r="K18" s="4">
+      <c r="K18" s="3">
         <v>1694599</v>
       </c>
       <c r="M18" s="1">
@@ -1082,16 +1034,13 @@
         <v>0</v>
       </c>
       <c r="O18" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P18" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q18" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="19" spans="7:17" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="P18" s="3">
+        <v>1694599</v>
+      </c>
+    </row>
+    <row r="19" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G19" s="1">
         <v>8</v>
       </c>
@@ -1104,7 +1053,7 @@
       <c r="J19" s="1">
         <v>12</v>
       </c>
-      <c r="K19" s="4">
+      <c r="K19" s="3">
         <v>304708</v>
       </c>
       <c r="M19" s="1">
@@ -1114,16 +1063,13 @@
         <v>1</v>
       </c>
       <c r="O19" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P19" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q19" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="20" spans="7:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P19" s="3">
+        <v>304708</v>
+      </c>
+    </row>
+    <row r="20" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G20" s="1">
         <v>8</v>
       </c>
@@ -1136,7 +1082,7 @@
       <c r="J20" s="1">
         <v>12</v>
       </c>
-      <c r="K20" s="4">
+      <c r="K20" s="3">
         <v>577915</v>
       </c>
       <c r="M20" s="1">
@@ -1146,16 +1092,13 @@
         <v>2</v>
       </c>
       <c r="O20" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P20" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q20" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="21" spans="7:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P20" s="3">
+        <v>577915</v>
+      </c>
+    </row>
+    <row r="21" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G21" s="1">
         <v>8</v>
       </c>
@@ -1168,7 +1111,7 @@
       <c r="J21" s="1">
         <v>8</v>
       </c>
-      <c r="K21" s="4">
+      <c r="K21" s="3">
         <v>1135200</v>
       </c>
       <c r="M21" s="1">
@@ -1178,16 +1121,13 @@
         <v>4</v>
       </c>
       <c r="O21" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P21" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q21" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="22" spans="7:17" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="P21" s="3">
+        <v>1135200</v>
+      </c>
+    </row>
+    <row r="22" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G22" s="1">
         <v>8</v>
       </c>
@@ -1200,7 +1140,7 @@
       <c r="J22" s="1">
         <v>6</v>
       </c>
-      <c r="K22" s="4">
+      <c r="K22" s="3">
         <v>1694599</v>
       </c>
       <c r="M22" s="1">
@@ -1210,16 +1150,13 @@
         <v>8</v>
       </c>
       <c r="O22" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P22" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q22" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="23" spans="7:17" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="P22" s="3">
+        <v>1694599</v>
+      </c>
+    </row>
+    <row r="23" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G23" s="1">
         <v>16</v>
       </c>
@@ -1232,7 +1169,7 @@
       <c r="J23" s="1">
         <v>6</v>
       </c>
-      <c r="K23" s="4">
+      <c r="K23" s="3">
         <v>1422675</v>
       </c>
       <c r="M23" s="1">
@@ -1242,16 +1179,13 @@
         <v>0</v>
       </c>
       <c r="O23" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P23" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q23" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="24" spans="7:17" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="P23" s="3">
+        <v>1422675</v>
+      </c>
+    </row>
+    <row r="24" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G24" s="1">
         <v>16</v>
       </c>
@@ -1264,7 +1198,7 @@
       <c r="J24" s="1">
         <v>12</v>
       </c>
-      <c r="K24" s="4">
+      <c r="K24" s="3">
         <v>304708</v>
       </c>
       <c r="M24" s="1">
@@ -1274,16 +1208,13 @@
         <v>1</v>
       </c>
       <c r="O24" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P24" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q24" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="25" spans="7:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P24" s="3">
+        <v>304708</v>
+      </c>
+    </row>
+    <row r="25" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G25" s="1">
         <v>16</v>
       </c>
@@ -1296,7 +1227,7 @@
       <c r="J25" s="1">
         <v>12</v>
       </c>
-      <c r="K25" s="4">
+      <c r="K25" s="3">
         <v>577915</v>
       </c>
       <c r="M25" s="1">
@@ -1306,16 +1237,13 @@
         <v>2</v>
       </c>
       <c r="O25" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P25" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q25" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="26" spans="7:17" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="P25" s="3">
+        <v>577915</v>
+      </c>
+    </row>
+    <row r="26" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G26" s="1">
         <v>16</v>
       </c>
@@ -1328,7 +1256,7 @@
       <c r="J26" s="1">
         <v>8</v>
       </c>
-      <c r="K26" s="4">
+      <c r="K26" s="3">
         <v>1135200</v>
       </c>
       <c r="M26" s="1">
@@ -1338,16 +1266,13 @@
         <v>4</v>
       </c>
       <c r="O26" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P26" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q26" s="4">
-        <v>160149</v>
-      </c>
-    </row>
-    <row r="27" spans="7:17" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="P26" s="3">
+        <v>1135200</v>
+      </c>
+    </row>
+    <row r="27" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G27" s="1">
         <v>16</v>
       </c>
@@ -1360,7 +1285,7 @@
       <c r="J27" s="1">
         <v>6</v>
       </c>
-      <c r="K27" s="4">
+      <c r="K27" s="3">
         <v>1422675</v>
       </c>
       <c r="M27" s="1">
@@ -1370,20 +1295,17 @@
         <v>8</v>
       </c>
       <c r="O27" s="1">
-        <v>87896</v>
-      </c>
-      <c r="P27" s="1">
-        <v>4</v>
-      </c>
-      <c r="Q27" s="4">
-        <v>160149</v>
+        <v>6</v>
+      </c>
+      <c r="P27" s="3">
+        <v>1422675</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="M1:Q1"/>
     <mergeCell ref="G1:K1"/>
+    <mergeCell ref="M1:P1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>